<commit_message>
Abänderungen, Verbesserungen, Bug Fixes & co.
</commit_message>
<xml_diff>
--- a/Prod/rpa002_DTJ_Performer_Prod_v02/Data/Config.xlsx
+++ b/Prod/rpa002_DTJ_Performer_Prod_v02/Data/Config.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26731"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27928"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ex.wosnitza\Documents\UiPath\Deutschlandticket\Data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\baris.isik\develop\rpa\uipath-rpa_dtj\Prod\rpa002_DTJ_Performer_Prod_v02\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ED539933-482A-4E81-A5ED-238A8CD36EA1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{237A09AE-BBBA-4DBB-9C7F-38BD51B563F4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" r:id="rId1"/>
@@ -152,9 +152,6 @@
     <t>D-Ticket</t>
   </si>
   <si>
-    <t>D-Ticket-Test-Queue</t>
-  </si>
-  <si>
     <t>Test\POR\rpa002_D-Ticket</t>
   </si>
   <si>
@@ -209,7 +206,10 @@
     <t>\\fsitm.muenchen.de\itm-ablage\Allgemein\RPA_Deutschlandticket_TEST\RPA_DTJ\Exceptions\Screenshots</t>
   </si>
   <si>
-    <t>rpa002_SAP-Account_K31</t>
+    <t>rpa002_SAP-Account</t>
+  </si>
+  <si>
+    <t>D-Ticket-Queue</t>
   </si>
 </sst>
 </file>
@@ -290,9 +290,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 – 2022-Design">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 – 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -330,7 +330,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 – 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -436,7 +436,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 – 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -578,7 +578,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -631,10 +631,10 @@
     </row>
     <row r="2" spans="1:26" ht="14.25" customHeight="1">
       <c r="A2" s="2" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>42</v>
+        <v>61</v>
       </c>
       <c r="C2" s="2" t="s">
         <v>20</v>
@@ -645,7 +645,7 @@
         <v>28</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C3" s="4" t="s">
         <v>29</v>
@@ -665,18 +665,18 @@
     </row>
     <row r="6" spans="1:26" ht="14.25" customHeight="1">
       <c r="A6" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B6" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="7" spans="1:26" ht="14.25" customHeight="1">
       <c r="A7" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B7" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="8" spans="1:26" ht="14.25" customHeight="1"/>
@@ -1750,7 +1750,7 @@
         <v>6</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C5" t="s">
         <v>7</v>
@@ -2884,122 +2884,122 @@
     </row>
     <row r="2" spans="1:26" ht="14.25" customHeight="1">
       <c r="A2" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B2" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="3" spans="1:26" ht="14.25" customHeight="1">
       <c r="A3" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B3" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="4" spans="1:26" ht="14.25" customHeight="1">
       <c r="A4" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B4" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="5" spans="1:26" ht="14.25" customHeight="1">
       <c r="A5" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B5" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="6" spans="1:26" ht="14.25" customHeight="1">
       <c r="A6" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B6" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="7" spans="1:26" ht="14.25" customHeight="1">
       <c r="A7" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B7" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="8" spans="1:26" ht="14.25" customHeight="1">
       <c r="A8" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B8" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="9" spans="1:26" ht="14.25" customHeight="1">
       <c r="A9" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B9" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
     <row r="10" spans="1:26" ht="14.25" customHeight="1">
       <c r="A10" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B10" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="11" spans="1:26" ht="14.25" customHeight="1">
       <c r="A11" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B11" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="12" spans="1:26" ht="14.25" customHeight="1">
       <c r="A12" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B12" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="13" spans="1:26" ht="14.25" customHeight="1">
       <c r="A13" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B13" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="14" spans="1:26" ht="14.25" customHeight="1">
       <c r="A14" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B14" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
     <row r="15" spans="1:26" ht="14.25" customHeight="1">
       <c r="A15" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B15" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
     </row>
     <row r="16" spans="1:26" ht="14.25" customHeight="1">
       <c r="A16" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B16" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="19" ht="14.25" customHeight="1"/>

</xml_diff>